<commit_message>
Updated test Excel file
</commit_message>
<xml_diff>
--- a/Testing_Docs/test1.xlsx
+++ b/Testing_Docs/test1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nikhi\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nishant\Final Year Project\Test\MultiDoc-ChatBot-main\Testing_Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE4BC1FA-A132-4DDB-B263-2E1DCB9984CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A83EEFFD-3CB1-44A3-928E-A623A96D301F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4272" yWindow="720" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -87,8 +87,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -373,49 +376,50 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="1">
         <v>30</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="1">
         <v>25</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="1">
         <v>35</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="1" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>